<commit_message>
update ATC db and update vragen.txt
</commit_message>
<xml_diff>
--- a/ATC_Groepen/ATC_groepen.xlsx
+++ b/ATC_Groepen/ATC_groepen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\semde\Documents\MedicatieReview\ATC_Groepen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF096BD7-AE82-4425-9522-6F31740559AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA7813D-1079-40C9-B7E1-240D41D09196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="14595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="212">
   <si>
     <t>ATC_groep</t>
   </si>
@@ -593,9 +593,6 @@
     <t>RLS</t>
   </si>
   <si>
-    <t>Epilepsie</t>
-  </si>
-  <si>
     <t>Parkinson</t>
   </si>
   <si>
@@ -671,10 +668,10 @@
     <t>Jansen_omschrijving</t>
   </si>
   <si>
-    <t>Gedragsbeïnvloedende geneesmiddelen</t>
-  </si>
-  <si>
     <t>Oren</t>
+  </si>
+  <si>
+    <t>Psychofarmaca</t>
   </si>
 </sst>
 </file>
@@ -1063,7 +1060,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
@@ -1195,7 +1192,7 @@
         <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.45">
@@ -1525,7 +1522,7 @@
         <v>85</v>
       </c>
       <c r="C43" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.45">
@@ -1536,7 +1533,7 @@
         <v>87</v>
       </c>
       <c r="C44" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.45">
@@ -1547,7 +1544,7 @@
         <v>89</v>
       </c>
       <c r="C45" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.45">
@@ -1558,7 +1555,7 @@
         <v>91</v>
       </c>
       <c r="C46" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.45">
@@ -1569,7 +1566,7 @@
         <v>93</v>
       </c>
       <c r="C47" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.45">
@@ -1591,7 +1588,7 @@
         <v>97</v>
       </c>
       <c r="C49" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.45">
@@ -1602,7 +1599,7 @@
         <v>99</v>
       </c>
       <c r="C50" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.45">
@@ -1613,7 +1610,7 @@
         <v>101</v>
       </c>
       <c r="C51" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.45">
@@ -1624,7 +1621,7 @@
         <v>103</v>
       </c>
       <c r="C52" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.45">
@@ -1635,7 +1632,7 @@
         <v>105</v>
       </c>
       <c r="C53" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.45">
@@ -1646,7 +1643,7 @@
         <v>107</v>
       </c>
       <c r="C54" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.45">
@@ -1657,7 +1654,7 @@
         <v>109</v>
       </c>
       <c r="C55" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.45">
@@ -1668,7 +1665,7 @@
         <v>111</v>
       </c>
       <c r="C56" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.45">
@@ -1679,7 +1676,7 @@
         <v>113</v>
       </c>
       <c r="C57" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.45">
@@ -1712,7 +1709,7 @@
         <v>119</v>
       </c>
       <c r="C60" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.45">
@@ -1778,7 +1775,7 @@
         <v>131</v>
       </c>
       <c r="C66" t="s">
-        <v>185</v>
+        <v>211</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.45">
@@ -1789,7 +1786,7 @@
         <v>133</v>
       </c>
       <c r="C67" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.45">
@@ -1833,7 +1830,7 @@
         <v>141</v>
       </c>
       <c r="C71" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.45">
@@ -1844,7 +1841,7 @@
         <v>143</v>
       </c>
       <c r="C72" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.45">
@@ -1866,7 +1863,7 @@
         <v>147</v>
       </c>
       <c r="C74" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.45">
@@ -1888,7 +1885,7 @@
         <v>151</v>
       </c>
       <c r="C76" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.45">
@@ -1899,7 +1896,7 @@
         <v>153</v>
       </c>
       <c r="C77" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.45">
@@ -1910,7 +1907,7 @@
         <v>155</v>
       </c>
       <c r="C78" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.45">
@@ -1921,7 +1918,7 @@
         <v>157</v>
       </c>
       <c r="C79" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.45">
@@ -1932,7 +1929,7 @@
         <v>159</v>
       </c>
       <c r="C80" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.45">
@@ -1943,7 +1940,7 @@
         <v>161</v>
       </c>
       <c r="C81" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.45">
@@ -1954,7 +1951,7 @@
         <v>163</v>
       </c>
       <c r="C82" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.45">

</xml_diff>